<commit_message>
movimiento del 2198 a fa6
</commit_message>
<xml_diff>
--- a/backend/data/AutomatedLines.xlsx
+++ b/backend/data/AutomatedLines.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kochind-my.sharepoint.com/personal/moises_ramirez1_molex_com/Documents/aplicacionWeb/WebAppLineFinder/backend/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="652" documentId="13_ncr:1_{9CF0DDEB-C0A7-4BC9-A395-14399483BEE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F3A0375F-9763-4D84-8668-0AD826C40505}"/>
+  <xr:revisionPtr revIDLastSave="654" documentId="13_ncr:1_{9CF0DDEB-C0A7-4BC9-A395-14399483BEE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFD0ED34-7814-4203-AC5A-E0ABCAD236EB}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1340,7 +1340,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2787,24 +2787,24 @@
     </dxf>
     <dxf>
       <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
         <bottom style="thin">
           <color auto="1"/>
         </bottom>
       </border>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -3029,7 +3029,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2551586D-350A-4849-A83B-B0EC7C8A022F}" name="Tabla2" displayName="Tabla2" ref="A1:CX10" totalsRowShown="0" headerRowDxfId="116" dataDxfId="115" headerRowBorderDxfId="113" tableBorderDxfId="114">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2551586D-350A-4849-A83B-B0EC7C8A022F}" name="Tabla2" displayName="Tabla2" ref="A1:CX10" totalsRowShown="0" headerRowDxfId="116" dataDxfId="114" headerRowBorderDxfId="115" tableBorderDxfId="113">
   <autoFilter ref="A1:CX10" xr:uid="{2551586D-350A-4849-A83B-B0EC7C8A022F}"/>
   <tableColumns count="102">
     <tableColumn id="1" xr3:uid="{515ED9AD-2115-402D-A669-A7974119647C}" name="Col 1" dataDxfId="112"/>
@@ -3475,19 +3475,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H233"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.85546875" customWidth="1"/>
+    <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.81640625" customWidth="1"/>
     <col min="3" max="3" width="15" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.81640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
@@ -3513,7 +3513,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2088701244</v>
       </c>
@@ -3527,7 +3527,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2088701390</v>
       </c>
@@ -3541,7 +3541,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2088701610</v>
       </c>
@@ -3555,7 +3555,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2088701746</v>
       </c>
@@ -3566,7 +3566,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2088702198</v>
       </c>
@@ -3580,7 +3580,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>2088702199</v>
       </c>
@@ -3594,7 +3594,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2088702200</v>
       </c>
@@ -3608,7 +3608,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>2088702201</v>
       </c>
@@ -3625,7 +3625,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>2088702202</v>
       </c>
@@ -3639,7 +3639,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>2088702203</v>
       </c>
@@ -3653,7 +3653,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>2088702204</v>
       </c>
@@ -3667,7 +3667,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>2088702205</v>
       </c>
@@ -3681,7 +3681,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>2088702206</v>
       </c>
@@ -3695,7 +3695,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>2088702207</v>
       </c>
@@ -3721,7 +3721,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>2088702221</v>
       </c>
@@ -3735,7 +3735,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>2088702318</v>
       </c>
@@ -3749,7 +3749,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>2088707042</v>
       </c>
@@ -3763,7 +3763,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>2098700024</v>
       </c>
@@ -3777,7 +3777,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20" s="5">
         <v>2098700025</v>
       </c>
@@ -3791,7 +3791,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>2098700026</v>
       </c>
@@ -3805,7 +3805,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>2098700033</v>
       </c>
@@ -3819,7 +3819,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>2098700046</v>
       </c>
@@ -3833,7 +3833,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>2098700056</v>
       </c>
@@ -3847,7 +3847,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>2098700058</v>
       </c>
@@ -3861,7 +3861,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>2098700076</v>
       </c>
@@ -3875,7 +3875,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>2098700083</v>
       </c>
@@ -3889,7 +3889,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28" s="5">
         <v>2098700108</v>
       </c>
@@ -3903,7 +3903,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>2098700143</v>
       </c>
@@ -3917,7 +3917,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>2098700154</v>
       </c>
@@ -3931,7 +3931,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="31" spans="1:4">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>2098700177</v>
       </c>
@@ -3945,7 +3945,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>2098700189</v>
       </c>
@@ -3959,7 +3959,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>2098700245</v>
       </c>
@@ -3973,7 +3973,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="34" spans="1:5">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="5">
         <v>2098700246</v>
       </c>
@@ -3987,7 +3987,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="35" spans="1:5">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="5">
         <v>2098700256</v>
       </c>
@@ -4001,7 +4001,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:5">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>2098700289</v>
       </c>
@@ -4015,7 +4015,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="37" spans="1:5">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>2098700290</v>
       </c>
@@ -4029,7 +4029,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="38" spans="1:5">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>2098700293</v>
       </c>
@@ -4043,7 +4043,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="39" spans="1:5">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>2098700296</v>
       </c>
@@ -4060,7 +4060,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="40" spans="1:5">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>2098700301</v>
       </c>
@@ -4074,7 +4074,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:5">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>2098700302</v>
       </c>
@@ -4088,7 +4088,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="42" spans="1:5">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>2098700304</v>
       </c>
@@ -4102,7 +4102,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>2098700305</v>
       </c>
@@ -4116,7 +4116,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>2098700306</v>
       </c>
@@ -4130,7 +4130,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>2098700307</v>
       </c>
@@ -4144,7 +4144,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>2098700309</v>
       </c>
@@ -4158,7 +4158,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>2098700315</v>
       </c>
@@ -4172,7 +4172,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>2098700316</v>
       </c>
@@ -4186,7 +4186,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="49" spans="1:4">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>2098700320</v>
       </c>
@@ -4200,7 +4200,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="50" spans="1:4">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>2098700322</v>
       </c>
@@ -4214,7 +4214,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="51" spans="1:4">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>2098700353</v>
       </c>
@@ -4228,7 +4228,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="52" spans="1:4">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>2098700355</v>
       </c>
@@ -4242,7 +4242,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="53" spans="1:4">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>2098700356</v>
       </c>
@@ -4256,7 +4256,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="54" spans="1:4">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>2098700357</v>
       </c>
@@ -4270,7 +4270,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="55" spans="1:4">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>2098700358</v>
       </c>
@@ -4284,7 +4284,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="56" spans="1:4">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>2098700366</v>
       </c>
@@ -4298,7 +4298,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="57" spans="1:4">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>2098700371</v>
       </c>
@@ -4312,7 +4312,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="58" spans="1:4">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>2098700372</v>
       </c>
@@ -4326,7 +4326,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="59" spans="1:4">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>2098700373</v>
       </c>
@@ -4340,7 +4340,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="60" spans="1:4">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>2098700374</v>
       </c>
@@ -4354,7 +4354,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="61" spans="1:4">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>2098700375</v>
       </c>
@@ -4368,7 +4368,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="62" spans="1:4">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>2098700376</v>
       </c>
@@ -4382,7 +4382,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="63" spans="1:4">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>2098700378</v>
       </c>
@@ -4396,7 +4396,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="64" spans="1:4">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" s="5">
         <v>2098700379</v>
       </c>
@@ -4410,7 +4410,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="65" spans="1:5">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A65" s="5">
         <v>2098700380</v>
       </c>
@@ -4424,7 +4424,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="66" spans="1:5">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A66" s="5">
         <v>2098700404</v>
       </c>
@@ -4438,7 +4438,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="67" spans="1:5">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A67" s="5">
         <v>2098700405</v>
       </c>
@@ -4452,7 +4452,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="68" spans="1:5">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>2098700429</v>
       </c>
@@ -4466,7 +4466,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="69" spans="1:5">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A69" s="5">
         <v>2098700432</v>
       </c>
@@ -4480,7 +4480,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="70" spans="1:5">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A70" s="5">
         <v>2098700433</v>
       </c>
@@ -4494,7 +4494,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="71" spans="1:5">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A71" s="5">
         <v>2098700434</v>
       </c>
@@ -4508,7 +4508,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="72" spans="1:5">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A72" s="5">
         <v>2098700436</v>
       </c>
@@ -4522,7 +4522,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="73" spans="1:5">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A73" s="5">
         <v>2098700437</v>
       </c>
@@ -4539,7 +4539,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="74" spans="1:5">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>2098701682</v>
       </c>
@@ -4553,7 +4553,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="75" spans="1:5">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>2098706005</v>
       </c>
@@ -4567,7 +4567,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="76" spans="1:5">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>2098706008</v>
       </c>
@@ -4581,7 +4581,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="77" spans="1:5">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>2098706009</v>
       </c>
@@ -4595,7 +4595,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="78" spans="1:5">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>2098706010</v>
       </c>
@@ -4609,7 +4609,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" spans="1:5">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>2098706011</v>
       </c>
@@ -4623,7 +4623,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="80" spans="1:5">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>2098706013</v>
       </c>
@@ -4637,7 +4637,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="81" spans="1:4">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>2098706018</v>
       </c>
@@ -4651,7 +4651,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="82" spans="1:4">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>2098706021</v>
       </c>
@@ -4665,7 +4665,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="83" spans="1:4">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>2098706023</v>
       </c>
@@ -4679,7 +4679,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="84" spans="1:4">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>2098706024</v>
       </c>
@@ -4693,7 +4693,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="85" spans="1:4">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>2098706025</v>
       </c>
@@ -4707,7 +4707,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="86" spans="1:4">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>2098706026</v>
       </c>
@@ -4721,7 +4721,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="87" spans="1:4">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>2098706028</v>
       </c>
@@ -4735,7 +4735,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="88" spans="1:4">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>2098706031</v>
       </c>
@@ -4749,7 +4749,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="89" spans="1:4">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>2098706032</v>
       </c>
@@ -4763,7 +4763,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="90" spans="1:4">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>2098706040</v>
       </c>
@@ -4777,7 +4777,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="91" spans="1:4">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>2098706041</v>
       </c>
@@ -4791,7 +4791,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="92" spans="1:4">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>2098706044</v>
       </c>
@@ -4805,7 +4805,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="93" spans="1:4">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A93" s="5">
         <v>2098706072</v>
       </c>
@@ -4819,7 +4819,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="94" spans="1:4">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A94" s="5">
         <v>2098706075</v>
       </c>
@@ -4833,7 +4833,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="95" spans="1:4">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95" s="5">
         <v>2098706076</v>
       </c>
@@ -4847,7 +4847,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="96" spans="1:4">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>2098706083</v>
       </c>
@@ -4861,7 +4861,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="97" spans="1:7">
+    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>2098706084</v>
       </c>
@@ -4875,7 +4875,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="98" spans="1:7">
+    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>2098706085</v>
       </c>
@@ -4889,7 +4889,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="99" spans="1:7">
+    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A99" s="5">
         <v>2098706087</v>
       </c>
@@ -4903,7 +4903,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="100" spans="1:7">
+    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A100" s="5">
         <v>2098706089</v>
       </c>
@@ -4917,7 +4917,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="101" spans="1:7">
+    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A101" s="5">
         <v>2099700009</v>
       </c>
@@ -4931,7 +4931,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="102" spans="1:7">
+    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A102" s="5">
         <v>2099700010</v>
       </c>
@@ -4945,7 +4945,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="103" spans="1:7">
+    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>2099700025</v>
       </c>
@@ -4962,7 +4962,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="104" spans="1:7">
+    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>2099700030</v>
       </c>
@@ -4982,7 +4982,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="105" spans="1:7">
+    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A105" s="5">
         <v>2099700041</v>
       </c>
@@ -4996,7 +4996,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="106" spans="1:7">
+    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A106">
         <v>2099700048</v>
       </c>
@@ -5010,7 +5010,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="107" spans="1:7">
+    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A107" s="5">
         <v>2099700049</v>
       </c>
@@ -5024,7 +5024,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="108" spans="1:7">
+    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A108" s="5">
         <v>2099700056</v>
       </c>
@@ -5038,7 +5038,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="109" spans="1:7">
+    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A109" s="5">
         <v>2099700057</v>
       </c>
@@ -5055,7 +5055,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="110" spans="1:7">
+    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A110" s="5">
         <v>2099700058</v>
       </c>
@@ -5078,7 +5078,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="111" spans="1:7">
+    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A111" s="5">
         <v>2099700059</v>
       </c>
@@ -5101,7 +5101,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="112" spans="1:7">
+    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A112" s="5">
         <v>2099706005</v>
       </c>
@@ -5115,7 +5115,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="113" spans="1:4">
+    <row r="113" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A113" s="5">
         <v>2154140069</v>
       </c>
@@ -5129,7 +5129,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="114" spans="1:4">
+    <row r="114" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A114" s="5">
         <v>2154140162</v>
       </c>
@@ -5143,7 +5143,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="115" spans="1:4">
+    <row r="115" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A115" s="5">
         <v>2154140207</v>
       </c>
@@ -5157,7 +5157,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="116" spans="1:4">
+    <row r="116" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A116">
         <v>2154140222</v>
       </c>
@@ -5171,7 +5171,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="117" spans="1:4">
+    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A117">
         <v>2154140224</v>
       </c>
@@ -5185,7 +5185,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="118" spans="1:4">
+    <row r="118" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A118">
         <v>2154140225</v>
       </c>
@@ -5199,7 +5199,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="119" spans="1:4">
+    <row r="119" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A119">
         <v>2154140229</v>
       </c>
@@ -5213,7 +5213,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="120" spans="1:4">
+    <row r="120" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A120">
         <v>2154140243</v>
       </c>
@@ -5227,7 +5227,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="121" spans="1:4">
+    <row r="121" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A121">
         <v>2154140283</v>
       </c>
@@ -5241,7 +5241,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="122" spans="1:4">
+    <row r="122" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A122">
         <v>2154140284</v>
       </c>
@@ -5255,7 +5255,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="123" spans="1:4">
+    <row r="123" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A123" s="5">
         <v>2154140285</v>
       </c>
@@ -5269,7 +5269,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="124" spans="1:4">
+    <row r="124" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A124">
         <v>2154140287</v>
       </c>
@@ -5283,7 +5283,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="125" spans="1:4">
+    <row r="125" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A125">
         <v>2154140289</v>
       </c>
@@ -5297,7 +5297,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="126" spans="1:4">
+    <row r="126" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A126">
         <v>2154140290</v>
       </c>
@@ -5311,7 +5311,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="127" spans="1:4">
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A127" s="5">
         <v>2154140291</v>
       </c>
@@ -5325,7 +5325,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="128" spans="1:4">
+    <row r="128" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A128" s="5">
         <v>2154140292</v>
       </c>
@@ -5339,7 +5339,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="129" spans="1:4">
+    <row r="129" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A129">
         <v>2154140293</v>
       </c>
@@ -5353,7 +5353,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="130" spans="1:4">
+    <row r="130" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A130">
         <v>2154140294</v>
       </c>
@@ -5367,7 +5367,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="131" spans="1:4">
+    <row r="131" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A131">
         <v>2154140295</v>
       </c>
@@ -5381,7 +5381,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="132" spans="1:4">
+    <row r="132" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A132">
         <v>2154140318</v>
       </c>
@@ -5395,7 +5395,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="133" spans="1:4">
+    <row r="133" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A133">
         <v>2154140319</v>
       </c>
@@ -5409,7 +5409,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="134" spans="1:4">
+    <row r="134" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A134" s="5">
         <v>2154140335</v>
       </c>
@@ -5423,7 +5423,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="135" spans="1:4">
+    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A135">
         <v>2154140336</v>
       </c>
@@ -5437,7 +5437,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="136" spans="1:4">
+    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A136" s="5">
         <v>2154140345</v>
       </c>
@@ -5451,7 +5451,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="137" spans="1:4">
+    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A137">
         <v>2154140349</v>
       </c>
@@ -5465,7 +5465,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="138" spans="1:4">
+    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A138" s="5">
         <v>2154140596</v>
       </c>
@@ -5479,7 +5479,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="139" spans="1:4">
+    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A139">
         <v>2154150035</v>
       </c>
@@ -5493,7 +5493,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="140" spans="1:4">
+    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A140">
         <v>2154150089</v>
       </c>
@@ -5507,7 +5507,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="141" spans="1:4">
+    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A141">
         <v>2154150163</v>
       </c>
@@ -5521,7 +5521,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="142" spans="1:4">
+    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A142">
         <v>2154150172</v>
       </c>
@@ -5535,7 +5535,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="143" spans="1:4">
+    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A143">
         <v>2154150197</v>
       </c>
@@ -5549,7 +5549,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="144" spans="1:4">
+    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A144">
         <v>2154150214</v>
       </c>
@@ -5563,7 +5563,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="145" spans="1:5">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A145">
         <v>2154150215</v>
       </c>
@@ -5577,7 +5577,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="146" spans="1:5">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A146">
         <v>2154150247</v>
       </c>
@@ -5591,7 +5591,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="147" spans="1:5">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A147">
         <v>2154150250</v>
       </c>
@@ -5605,7 +5605,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="148" spans="1:5">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A148" s="5">
         <v>2154150301</v>
       </c>
@@ -5619,7 +5619,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="149" spans="1:5">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A149">
         <v>2154150337</v>
       </c>
@@ -5633,7 +5633,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="150" spans="1:5">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A150">
         <v>2154150341</v>
       </c>
@@ -5647,7 +5647,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="151" spans="1:5">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A151">
         <v>2154150342</v>
       </c>
@@ -5661,7 +5661,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="152" spans="1:5">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A152" s="5">
         <v>2154150343</v>
       </c>
@@ -5675,7 +5675,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="153" spans="1:5">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A153" s="5">
         <v>2154150347</v>
       </c>
@@ -5689,7 +5689,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="154" spans="1:5">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A154">
         <v>2154150348</v>
       </c>
@@ -5703,7 +5703,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="155" spans="1:5">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A155" s="5">
         <v>2154150349</v>
       </c>
@@ -5717,7 +5717,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="156" spans="1:5">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A156" s="5">
         <v>2154150350</v>
       </c>
@@ -5734,7 +5734,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="157" spans="1:5">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A157" s="5">
         <v>2154150351</v>
       </c>
@@ -5748,7 +5748,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="158" spans="1:5">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A158" s="5">
         <v>2154150357</v>
       </c>
@@ -5765,7 +5765,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="159" spans="1:5">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A159" s="5">
         <v>2154150358</v>
       </c>
@@ -5779,7 +5779,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="160" spans="1:5">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A160" s="5">
         <v>2154150366</v>
       </c>
@@ -5796,7 +5796,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="161" spans="1:5">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A161" s="5">
         <v>2154150370</v>
       </c>
@@ -5810,7 +5810,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="162" spans="1:5">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A162">
         <v>2154150380</v>
       </c>
@@ -5824,7 +5824,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="163" spans="1:5">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A163">
         <v>2154150391</v>
       </c>
@@ -5838,7 +5838,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="164" spans="1:5">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A164">
         <v>2154150420</v>
       </c>
@@ -5852,7 +5852,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="165" spans="1:5">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A165">
         <v>2154150447</v>
       </c>
@@ -5866,7 +5866,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="166" spans="1:5">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A166" s="5">
         <v>2154150448</v>
       </c>
@@ -5880,7 +5880,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="167" spans="1:5">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A167" s="5">
         <v>2154150455</v>
       </c>
@@ -5897,7 +5897,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="168" spans="1:5">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A168">
         <v>2154150461</v>
       </c>
@@ -5911,7 +5911,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="169" spans="1:5">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A169" s="5">
         <v>2154150497</v>
       </c>
@@ -5925,7 +5925,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="170" spans="1:5">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A170" s="5">
         <v>2154150501</v>
       </c>
@@ -5939,7 +5939,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="171" spans="1:5">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A171" s="5">
         <v>2154150509</v>
       </c>
@@ -5953,7 +5953,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="172" spans="1:5">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A172" s="5">
         <v>2154150525</v>
       </c>
@@ -5970,7 +5970,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="173" spans="1:5">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A173" s="5">
         <v>2154150526</v>
       </c>
@@ -5984,7 +5984,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="174" spans="1:5">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A174" s="5">
         <v>2154150534</v>
       </c>
@@ -6001,7 +6001,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="175" spans="1:5">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A175">
         <v>2154150554</v>
       </c>
@@ -6015,7 +6015,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="176" spans="1:5">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A176" s="5">
         <v>2154150557</v>
       </c>
@@ -6029,7 +6029,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="177" spans="1:6">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A177" s="5">
         <v>2154150560</v>
       </c>
@@ -6049,7 +6049,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="178" spans="1:6">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A178">
         <v>2154150563</v>
       </c>
@@ -6063,7 +6063,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="179" spans="1:6">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A179" s="5">
         <v>2154150581</v>
       </c>
@@ -6077,7 +6077,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="180" spans="1:6">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A180">
         <v>2154150582</v>
       </c>
@@ -6091,7 +6091,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="181" spans="1:6">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A181">
         <v>2154150588</v>
       </c>
@@ -6105,7 +6105,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="182" spans="1:6">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A182" s="5">
         <v>2154150591</v>
       </c>
@@ -6122,7 +6122,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="183" spans="1:6">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A183" s="5">
         <v>2154150597</v>
       </c>
@@ -6139,7 +6139,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="184" spans="1:6">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A184">
         <v>2154150603</v>
       </c>
@@ -6153,7 +6153,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="185" spans="1:6">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A185">
         <v>2154150605</v>
       </c>
@@ -6167,7 +6167,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="186" spans="1:6">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A186" s="5">
         <v>2154150622</v>
       </c>
@@ -6181,7 +6181,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="187" spans="1:6">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A187" s="5">
         <v>2154150627</v>
       </c>
@@ -6195,7 +6195,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="188" spans="1:6">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A188">
         <v>2154150633</v>
       </c>
@@ -6209,7 +6209,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="189" spans="1:6">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A189" s="5">
         <v>2154150646</v>
       </c>
@@ -6229,7 +6229,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="190" spans="1:6">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A190" s="5">
         <v>2154150648</v>
       </c>
@@ -6249,7 +6249,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="191" spans="1:6">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A191" s="5">
         <v>2154150653</v>
       </c>
@@ -6263,7 +6263,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="192" spans="1:6">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A192">
         <v>2154150669</v>
       </c>
@@ -6277,7 +6277,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="193" spans="1:6">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A193">
         <v>2154150672</v>
       </c>
@@ -6291,7 +6291,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="194" spans="1:6">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A194" s="5">
         <v>2154150677</v>
       </c>
@@ -6308,7 +6308,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="195" spans="1:6">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A195">
         <v>2154150706</v>
       </c>
@@ -6322,7 +6322,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="196" spans="1:6">
+    <row r="196" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A196">
         <v>2154150707</v>
       </c>
@@ -6336,7 +6336,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="197" spans="1:6">
+    <row r="197" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A197">
         <v>2154150715</v>
       </c>
@@ -6350,7 +6350,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="198" spans="1:6">
+    <row r="198" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A198" s="5">
         <v>2154150719</v>
       </c>
@@ -6364,7 +6364,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="199" spans="1:6">
+    <row r="199" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A199" s="5">
         <v>2154150731</v>
       </c>
@@ -6378,7 +6378,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="200" spans="1:6">
+    <row r="200" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A200" s="5">
         <v>2154150765</v>
       </c>
@@ -6398,7 +6398,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="201" spans="1:6">
+    <row r="201" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A201" s="5">
         <v>2154150767</v>
       </c>
@@ -6418,7 +6418,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="202" spans="1:6">
+    <row r="202" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A202" s="5">
         <v>2154150769</v>
       </c>
@@ -6435,7 +6435,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="203" spans="1:6">
+    <row r="203" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A203" s="5">
         <v>2154150788</v>
       </c>
@@ -6449,7 +6449,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="204" spans="1:6">
+    <row r="204" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A204" s="5">
         <v>2154150813</v>
       </c>
@@ -6469,7 +6469,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="205" spans="1:6">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A205" s="5">
         <v>2154150814</v>
       </c>
@@ -6486,7 +6486,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="206" spans="1:6">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A206" s="5">
         <v>2154150822</v>
       </c>
@@ -6503,7 +6503,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="207" spans="1:6">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A207" s="5">
         <v>2154150839</v>
       </c>
@@ -6517,7 +6517,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="208" spans="1:6">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A208" s="5">
         <v>2154150840</v>
       </c>
@@ -6531,7 +6531,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="209" spans="1:5">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A209" s="5">
         <v>2154150841</v>
       </c>
@@ -6545,7 +6545,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="210" spans="1:5">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A210" s="5">
         <v>2154150876</v>
       </c>
@@ -6559,7 +6559,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="211" spans="1:5">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A211" s="5">
         <v>2154150893</v>
       </c>
@@ -6573,7 +6573,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="212" spans="1:5">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A212" s="5">
         <v>2154150918</v>
       </c>
@@ -6587,7 +6587,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="213" spans="1:5">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A213" s="5">
         <v>2154150921</v>
       </c>
@@ -6601,7 +6601,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="214" spans="1:5">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A214" s="5">
         <v>2154150922</v>
       </c>
@@ -6615,7 +6615,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="215" spans="1:5">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A215">
         <v>2154150943</v>
       </c>
@@ -6629,7 +6629,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="216" spans="1:5">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A216">
         <v>2154155136</v>
       </c>
@@ -6643,7 +6643,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="217" spans="1:5">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A217" s="5">
         <v>2154155149</v>
       </c>
@@ -6657,7 +6657,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="218" spans="1:5">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A218" s="5">
         <v>2154155150</v>
       </c>
@@ -6674,7 +6674,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="219" spans="1:5">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A219">
         <v>2154160029</v>
       </c>
@@ -6688,7 +6688,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="220" spans="1:5">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A220">
         <v>2154160030</v>
       </c>
@@ -6702,7 +6702,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="221" spans="1:5">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A221">
         <v>2154160031</v>
       </c>
@@ -6716,7 +6716,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="222" spans="1:5">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A222">
         <v>2154160032</v>
       </c>
@@ -6730,7 +6730,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="223" spans="1:5">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A223">
         <v>2154160033</v>
       </c>
@@ -6744,7 +6744,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="224" spans="1:5">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A224">
         <v>2154160034</v>
       </c>
@@ -6758,7 +6758,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="225" spans="1:7">
+    <row r="225" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A225">
         <v>2154160035</v>
       </c>
@@ -6772,7 +6772,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="226" spans="1:7">
+    <row r="226" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A226" s="5">
         <v>2154160036</v>
       </c>
@@ -6786,7 +6786,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="227" spans="1:7">
+    <row r="227" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A227">
         <v>2154160037</v>
       </c>
@@ -6800,7 +6800,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="228" spans="1:7">
+    <row r="228" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A228">
         <v>2154170049</v>
       </c>
@@ -6814,7 +6814,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="229" spans="1:7">
+    <row r="229" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A229">
         <v>2154170050</v>
       </c>
@@ -6837,7 +6837,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="230" spans="1:7">
+    <row r="230" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A230">
         <v>2154170052</v>
       </c>
@@ -6851,7 +6851,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="233" spans="1:7">
+    <row r="233" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A233" s="5"/>
       <c r="B233" s="5"/>
     </row>
@@ -6871,88 +6871,88 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:CX10"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="9.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.7109375" style="39" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="13.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.28515625" style="39" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="13.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.7109375" style="39" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.5703125" style="39" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.85546875" style="39" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.28515625" style="39" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.5703125" style="39" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.7109375" style="39" bestFit="1" customWidth="1"/>
-    <col min="16" max="17" width="13.85546875" style="39" bestFit="1" customWidth="1"/>
-    <col min="18" max="19" width="13.7109375" style="39" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="9.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.7265625" style="39" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="13.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.26953125" style="39" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="13.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.7265625" style="39" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.54296875" style="39" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.81640625" style="39" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.26953125" style="39" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="13.54296875" style="39" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.7265625" style="39" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="13.81640625" style="39" bestFit="1" customWidth="1"/>
+    <col min="18" max="19" width="13.7265625" style="39" bestFit="1" customWidth="1"/>
     <col min="20" max="21" width="14" style="39" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="13.85546875" style="39" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="16.5703125" style="39" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="13.5703125" style="39" bestFit="1" customWidth="1"/>
-    <col min="26" max="27" width="13.28515625" style="39" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="13.7109375" style="39" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="13.85546875" style="39" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" style="39" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="13.5703125" style="39" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="14.5703125" style="39" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="13.85546875" style="39" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="12.28515625" style="39" bestFit="1" customWidth="1"/>
-    <col min="37" max="38" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="11.42578125" style="39" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.81640625" style="39" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="16.54296875" style="39" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="13.54296875" style="39" bestFit="1" customWidth="1"/>
+    <col min="26" max="27" width="13.26953125" style="39" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="13.7265625" style="39" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="13.81640625" style="39" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12.81640625" style="39" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="13.54296875" style="39" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="14.54296875" style="39" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="13.81640625" style="39" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="12.26953125" style="39" bestFit="1" customWidth="1"/>
+    <col min="37" max="38" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="11.453125" style="39" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="12" style="39" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="12.140625" style="39" bestFit="1" customWidth="1"/>
-    <col min="43" max="44" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="12.5703125" style="39" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="12.7109375" style="39" bestFit="1" customWidth="1"/>
-    <col min="47" max="48" width="12.85546875" style="39" bestFit="1" customWidth="1"/>
-    <col min="49" max="49" width="12.7109375" style="39" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="12.5703125" style="39" bestFit="1" customWidth="1"/>
-    <col min="51" max="51" width="12.85546875" style="39" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="12.7109375" style="39" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="11.85546875" style="39" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="55" max="55" width="12.7109375" style="39" bestFit="1" customWidth="1"/>
-    <col min="56" max="56" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="57" max="57" width="12.85546875" style="39" bestFit="1" customWidth="1"/>
-    <col min="58" max="58" width="12.7109375" style="39" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="12.28515625" style="39" bestFit="1" customWidth="1"/>
-    <col min="60" max="63" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="64" max="64" width="12.28515625" style="39" bestFit="1" customWidth="1"/>
-    <col min="65" max="66" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="67" max="67" width="11.42578125" style="39" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="12.1796875" style="39" bestFit="1" customWidth="1"/>
+    <col min="43" max="44" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="12.54296875" style="39" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="12.7265625" style="39" bestFit="1" customWidth="1"/>
+    <col min="47" max="48" width="12.81640625" style="39" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="12.7265625" style="39" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="12.54296875" style="39" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="12.81640625" style="39" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="12.7265625" style="39" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="11.81640625" style="39" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="12.7265625" style="39" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="12.81640625" style="39" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="12.7265625" style="39" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="12.26953125" style="39" bestFit="1" customWidth="1"/>
+    <col min="60" max="63" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="12.26953125" style="39" bestFit="1" customWidth="1"/>
+    <col min="65" max="66" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="11.453125" style="39" bestFit="1" customWidth="1"/>
     <col min="68" max="68" width="12" style="39" bestFit="1" customWidth="1"/>
-    <col min="69" max="69" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="70" max="70" width="12.140625" style="39" bestFit="1" customWidth="1"/>
-    <col min="71" max="72" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="73" max="73" width="12.28515625" style="39" bestFit="1" customWidth="1"/>
-    <col min="74" max="77" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="78" max="78" width="12.28515625" style="39" bestFit="1" customWidth="1"/>
-    <col min="79" max="80" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="81" max="81" width="11.42578125" style="39" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="12.1796875" style="39" bestFit="1" customWidth="1"/>
+    <col min="71" max="72" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="73" max="73" width="12.26953125" style="39" bestFit="1" customWidth="1"/>
+    <col min="74" max="77" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="12.26953125" style="39" bestFit="1" customWidth="1"/>
+    <col min="79" max="80" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="11.453125" style="39" bestFit="1" customWidth="1"/>
     <col min="82" max="82" width="12" style="39" bestFit="1" customWidth="1"/>
-    <col min="83" max="83" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="84" max="84" width="12.140625" style="39" bestFit="1" customWidth="1"/>
-    <col min="85" max="86" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="87" max="87" width="12.28515625" style="39" bestFit="1" customWidth="1"/>
-    <col min="88" max="91" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="92" max="92" width="12.28515625" style="39" bestFit="1" customWidth="1"/>
-    <col min="93" max="94" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="95" max="95" width="11.42578125" style="39" bestFit="1" customWidth="1"/>
+    <col min="83" max="83" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="84" max="84" width="12.1796875" style="39" bestFit="1" customWidth="1"/>
+    <col min="85" max="86" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="87" max="87" width="12.26953125" style="39" bestFit="1" customWidth="1"/>
+    <col min="88" max="91" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="92" max="92" width="12.26953125" style="39" bestFit="1" customWidth="1"/>
+    <col min="93" max="94" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="95" max="95" width="11.453125" style="39" bestFit="1" customWidth="1"/>
     <col min="96" max="96" width="12" style="39" bestFit="1" customWidth="1"/>
-    <col min="97" max="97" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="98" max="98" width="12.140625" style="39" bestFit="1" customWidth="1"/>
-    <col min="99" max="100" width="12.42578125" style="39" bestFit="1" customWidth="1"/>
-    <col min="101" max="101" width="13.42578125" style="39" bestFit="1" customWidth="1"/>
+    <col min="97" max="97" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="98" max="98" width="12.1796875" style="39" bestFit="1" customWidth="1"/>
+    <col min="99" max="100" width="12.453125" style="39" bestFit="1" customWidth="1"/>
+    <col min="101" max="101" width="13.453125" style="39" bestFit="1" customWidth="1"/>
     <col min="102" max="102" width="13" style="39" bestFit="1" customWidth="1"/>
-    <col min="103" max="16384" width="8.7109375" style="39"/>
+    <col min="103" max="16384" width="8.7265625" style="39"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:102">
+    <row r="1" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
@@ -7260,7 +7260,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="2" spans="1:102">
+    <row r="2" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A2" s="39" t="s">
         <v>205</v>
       </c>
@@ -7568,7 +7568,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="3" spans="1:102">
+    <row r="3" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A3" s="39" t="s">
         <v>252</v>
       </c>
@@ -7603,7 +7603,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:102">
+    <row r="4" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A4" s="39" t="s">
         <v>254</v>
       </c>
@@ -7650,7 +7650,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:102">
+    <row r="5" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A5" s="39" t="s">
         <v>256</v>
       </c>
@@ -7721,37 +7721,34 @@
         <v>106</v>
       </c>
       <c r="X5" s="41" t="s">
-        <v>13</v>
+        <v>70</v>
       </c>
       <c r="Y5" s="41" t="s">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="Z5" s="41" t="s">
-        <v>30</v>
+        <v>66</v>
       </c>
       <c r="AA5" s="41" t="s">
-        <v>66</v>
+        <v>85</v>
       </c>
       <c r="AB5" s="41" t="s">
-        <v>85</v>
+        <v>39</v>
       </c>
       <c r="AC5" s="41" t="s">
-        <v>39</v>
-      </c>
-      <c r="AD5" s="41" t="s">
         <v>50</v>
       </c>
-      <c r="AE5" s="42" t="s">
+      <c r="AD5" s="42" t="s">
         <v>36</v>
       </c>
+      <c r="AE5" s="41" t="s">
+        <v>52</v>
+      </c>
       <c r="AF5" s="41" t="s">
-        <v>52</v>
-      </c>
-      <c r="AG5" s="41" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="6" spans="1:102">
+    <row r="6" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A6" s="39" t="s">
         <v>258</v>
       </c>
@@ -7843,7 +7840,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="7" spans="1:102">
+    <row r="7" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A7" s="39" t="s">
         <v>261</v>
       </c>
@@ -7910,8 +7907,11 @@
       <c r="V7" s="42" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="8" spans="1:102">
+      <c r="W7" s="41" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A8" s="39" t="s">
         <v>263</v>
       </c>
@@ -7972,7 +7972,7 @@
       <c r="T8" s="43"/>
       <c r="U8" s="43"/>
     </row>
-    <row r="9" spans="1:102">
+    <row r="9" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A9" s="39" t="s">
         <v>265</v>
       </c>
@@ -8016,7 +8016,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="10" spans="1:102">
+    <row r="10" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A10" s="39" t="s">
         <v>267</v>
       </c>
@@ -8132,13 +8132,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AZ11"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="52" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="52" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52">
+    <row r="1" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -8248,7 +8248,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="2" spans="1:52">
+    <row r="2" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>267</v>
       </c>
@@ -8296,7 +8296,7 @@
       <c r="AI2" s="36"/>
       <c r="AJ2" s="36"/>
     </row>
-    <row r="3" spans="1:52">
+    <row r="3" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>205</v>
       </c>
@@ -8403,7 +8403,7 @@
         <v>2098700189</v>
       </c>
     </row>
-    <row r="4" spans="1:52">
+    <row r="4" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>252</v>
       </c>
@@ -8459,7 +8459,7 @@
         <v>2154150715</v>
       </c>
     </row>
-    <row r="5" spans="1:52">
+    <row r="5" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>254</v>
       </c>
@@ -8524,7 +8524,7 @@
         <v>2098706010</v>
       </c>
     </row>
-    <row r="6" spans="1:52">
+    <row r="6" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>256</v>
       </c>
@@ -8613,7 +8613,7 @@
         <v>2088702198</v>
       </c>
     </row>
-    <row r="7" spans="1:52">
+    <row r="7" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>258</v>
       </c>
@@ -8771,7 +8771,7 @@
         <v>2088701390</v>
       </c>
     </row>
-    <row r="8" spans="1:52">
+    <row r="8" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>261</v>
       </c>
@@ -8851,7 +8851,7 @@
         <v>2088707042</v>
       </c>
     </row>
-    <row r="9" spans="1:52">
+    <row r="9" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>263</v>
       </c>
@@ -8895,7 +8895,7 @@
         <v>2098700437</v>
       </c>
     </row>
-    <row r="10" spans="1:52">
+    <row r="10" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>265</v>
       </c>
@@ -8921,7 +8921,7 @@
         <v>2154170049</v>
       </c>
     </row>
-    <row r="11" spans="1:52">
+    <row r="11" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>377</v>
       </c>
@@ -8934,12 +8934,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="66.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="66.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>378</v>
       </c>
@@ -8947,7 +8947,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>266</v>
       </c>
@@ -8955,7 +8955,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>257</v>
       </c>
@@ -8963,7 +8963,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>262</v>
       </c>
@@ -8971,7 +8971,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>383</v>
       </c>
@@ -8979,7 +8979,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>257</v>
       </c>
@@ -8987,7 +8987,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>386</v>
       </c>
@@ -8995,7 +8995,7 @@
         <v>387</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>266</v>
       </c>
@@ -9003,7 +9003,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>259</v>
       </c>
@@ -9011,7 +9011,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>257</v>
       </c>
@@ -9019,7 +9019,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>257</v>
       </c>
@@ -9027,7 +9027,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>257</v>
       </c>
@@ -9035,7 +9035,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>393</v>
       </c>
@@ -9043,7 +9043,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>268</v>
       </c>
@@ -9051,7 +9051,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>259</v>
       </c>
@@ -9067,17 +9067,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA531276-FCFB-48E9-A31C-F81A22563EEA}">
   <dimension ref="A1:J40"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15" thickBot="1">
+    <row r="1" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="6" t="s">
         <v>397</v>
       </c>
@@ -9106,7 +9106,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="15" thickBot="1">
+    <row r="2" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="9" t="s">
         <v>406</v>
       </c>
@@ -9135,7 +9135,7 @@
         <v>414</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="60">
+    <row r="3" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A3" s="12" t="s">
         <v>415</v>
       </c>
@@ -9167,7 +9167,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="60">
+    <row r="4" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A4" s="15" t="s">
         <v>416</v>
       </c>
@@ -9199,7 +9199,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="60">
+    <row r="5" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A5" s="15" t="s">
         <v>418</v>
       </c>
@@ -9231,7 +9231,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="80.099999999999994">
+    <row r="6" spans="1:10" ht="80" x14ac:dyDescent="0.35">
       <c r="A6" s="15" t="s">
         <v>419</v>
       </c>
@@ -9263,7 +9263,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="60">
+    <row r="7" spans="1:10" ht="60" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
         <v>421</v>
       </c>
@@ -9295,7 +9295,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="60">
+    <row r="8" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A8" s="15" t="s">
         <v>422</v>
       </c>
@@ -9327,7 +9327,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="60">
+    <row r="9" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A9" s="15" t="s">
         <v>423</v>
       </c>
@@ -9359,7 +9359,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="60">
+    <row r="10" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A10" s="15" t="s">
         <v>25</v>
       </c>
@@ -9389,7 +9389,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="60">
+    <row r="11" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A11" s="20"/>
       <c r="B11" s="19"/>
       <c r="C11" s="16" t="s">
@@ -9417,7 +9417,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="60">
+    <row r="12" spans="1:10" ht="60" x14ac:dyDescent="0.35">
       <c r="A12" s="20"/>
       <c r="B12" s="19"/>
       <c r="C12" s="16" t="s">
@@ -9445,7 +9445,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="60">
+    <row r="13" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A13" s="20"/>
       <c r="B13" s="19"/>
       <c r="C13" s="16" t="s">
@@ -9473,7 +9473,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="60">
+    <row r="14" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A14" s="20"/>
       <c r="B14" s="19"/>
       <c r="C14" s="19"/>
@@ -9499,7 +9499,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="60">
+    <row r="15" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A15" s="20"/>
       <c r="B15" s="19"/>
       <c r="C15" s="19"/>
@@ -9523,7 +9523,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="60">
+    <row r="16" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A16" s="20"/>
       <c r="B16" s="19"/>
       <c r="C16" s="19"/>
@@ -9547,7 +9547,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="60">
+    <row r="17" spans="1:10" ht="60" x14ac:dyDescent="0.35">
       <c r="A17" s="20"/>
       <c r="B17" s="19"/>
       <c r="C17" s="19"/>
@@ -9571,7 +9571,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="18" spans="1:10" ht="60">
+    <row r="18" spans="1:10" ht="60" x14ac:dyDescent="0.35">
       <c r="A18" s="20"/>
       <c r="B18" s="19"/>
       <c r="C18" s="19"/>
@@ -9595,7 +9595,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:10" ht="60">
+    <row r="19" spans="1:10" ht="60" x14ac:dyDescent="0.35">
       <c r="A19" s="20"/>
       <c r="B19" s="19"/>
       <c r="C19" s="19"/>
@@ -9619,7 +9619,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="60">
+    <row r="20" spans="1:10" ht="60" x14ac:dyDescent="0.35">
       <c r="A20" s="20"/>
       <c r="B20" s="19"/>
       <c r="C20" s="19"/>
@@ -9643,7 +9643,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="60">
+    <row r="21" spans="1:10" ht="60" x14ac:dyDescent="0.35">
       <c r="A21" s="20"/>
       <c r="B21" s="19"/>
       <c r="C21" s="19"/>
@@ -9667,7 +9667,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="22" spans="1:10" ht="60">
+    <row r="22" spans="1:10" ht="60" x14ac:dyDescent="0.35">
       <c r="A22" s="20"/>
       <c r="B22" s="19"/>
       <c r="C22" s="19"/>
@@ -9689,7 +9689,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="23" spans="1:10" ht="60">
+    <row r="23" spans="1:10" ht="60" x14ac:dyDescent="0.35">
       <c r="A23" s="20"/>
       <c r="B23" s="19"/>
       <c r="C23" s="19"/>
@@ -9711,7 +9711,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="24" spans="1:10" ht="60">
+    <row r="24" spans="1:10" ht="60" x14ac:dyDescent="0.35">
       <c r="A24" s="24"/>
       <c r="B24" s="25"/>
       <c r="C24" s="25"/>
@@ -9733,7 +9733,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="60">
+    <row r="25" spans="1:10" ht="60" x14ac:dyDescent="0.35">
       <c r="A25" s="24"/>
       <c r="B25" s="25"/>
       <c r="C25" s="25"/>
@@ -9755,7 +9755,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="60">
+    <row r="26" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A26" s="24"/>
       <c r="B26" s="25"/>
       <c r="C26" s="25"/>
@@ -9775,7 +9775,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="27" spans="1:10" ht="60">
+    <row r="27" spans="1:10" ht="60" x14ac:dyDescent="0.35">
       <c r="A27" s="24"/>
       <c r="B27" s="25"/>
       <c r="C27" s="25"/>
@@ -9795,7 +9795,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="28" spans="1:10" ht="60">
+    <row r="28" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A28" s="20"/>
       <c r="B28" s="19"/>
       <c r="C28" s="19"/>
@@ -9813,7 +9813,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="60">
+    <row r="29" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A29" s="20"/>
       <c r="B29" s="19"/>
       <c r="C29" s="19"/>
@@ -9831,7 +9831,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="30" spans="1:10" ht="60">
+    <row r="30" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A30" s="20"/>
       <c r="B30" s="19"/>
       <c r="C30" s="19"/>
@@ -9849,7 +9849,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="31" spans="1:10" ht="60">
+    <row r="31" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A31" s="20"/>
       <c r="B31" s="19"/>
       <c r="C31" s="19"/>
@@ -9867,7 +9867,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:10" ht="60">
+    <row r="32" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A32" s="20"/>
       <c r="B32" s="19"/>
       <c r="C32" s="19"/>
@@ -9885,7 +9885,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="33" spans="1:10" ht="60">
+    <row r="33" spans="1:10" ht="40" x14ac:dyDescent="0.35">
       <c r="A33" s="20"/>
       <c r="B33" s="19"/>
       <c r="C33" s="19"/>
@@ -9903,7 +9903,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="60">
+    <row r="34" spans="1:10" ht="60" x14ac:dyDescent="0.35">
       <c r="A34" s="20"/>
       <c r="B34" s="19"/>
       <c r="C34" s="19"/>
@@ -9919,7 +9919,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="35" spans="1:10">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35" s="20"/>
       <c r="B35" s="19"/>
       <c r="C35" s="19"/>
@@ -9932,7 +9932,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="36" spans="1:10">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36" s="20"/>
       <c r="B36" s="19"/>
       <c r="C36" s="19"/>
@@ -9945,7 +9945,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="37" spans="1:10">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37" s="20"/>
       <c r="B37" s="19"/>
       <c r="C37" s="19"/>
@@ -9958,7 +9958,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="38" spans="1:10">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38" s="20"/>
       <c r="B38" s="19"/>
       <c r="C38" s="19"/>
@@ -9971,7 +9971,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="39" spans="1:10">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39" s="20"/>
       <c r="B39" s="19"/>
       <c r="C39" s="19"/>
@@ -9984,7 +9984,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="15" thickBot="1">
+    <row r="40" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="30"/>
       <c r="B40" s="31"/>
       <c r="C40" s="31"/>
@@ -10008,16 +10008,16 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I101"/>
-  <sheetFormatPr defaultColWidth="13.140625" defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="13.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="8" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="5" max="8" width="13.453125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="22.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>205</v>
       </c>
@@ -10046,7 +10046,7 @@
         <v>377</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>206</v>
       </c>
@@ -10075,7 +10075,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -10104,7 +10104,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>207</v>
       </c>
@@ -10133,7 +10133,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -10162,7 +10162,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -10191,7 +10191,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>27</v>
       </c>
@@ -10220,7 +10220,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>30</v>
       </c>
@@ -10249,7 +10249,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>208</v>
       </c>
@@ -10278,7 +10278,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>209</v>
       </c>
@@ -10304,7 +10304,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>210</v>
       </c>
@@ -10330,7 +10330,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>211</v>
       </c>
@@ -10356,7 +10356,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>49</v>
       </c>
@@ -10382,7 +10382,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -10405,7 +10405,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>212</v>
       </c>
@@ -10428,7 +10428,7 @@
         <v>272</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>213</v>
       </c>
@@ -10451,7 +10451,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>214</v>
       </c>
@@ -10471,7 +10471,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>215</v>
       </c>
@@ -10491,7 +10491,7 @@
         <v>420</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>41</v>
       </c>
@@ -10511,7 +10511,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>43</v>
       </c>
@@ -10531,7 +10531,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>35</v>
       </c>
@@ -10551,7 +10551,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>14</v>
       </c>
@@ -10571,7 +10571,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>216</v>
       </c>
@@ -10588,7 +10588,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>217</v>
       </c>
@@ -10602,7 +10602,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>218</v>
       </c>
@@ -10616,7 +10616,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="26" spans="1:9">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>219</v>
       </c>
@@ -10627,7 +10627,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>220</v>
       </c>
@@ -10638,7 +10638,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>33</v>
       </c>
@@ -10649,7 +10649,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="29" spans="1:9">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>221</v>
       </c>
@@ -10660,7 +10660,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="30" spans="1:9">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>16</v>
       </c>
@@ -10671,7 +10671,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="31" spans="1:9">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>214</v>
       </c>
@@ -10682,7 +10682,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="32" spans="1:9">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>215</v>
       </c>
@@ -10693,7 +10693,7 @@
         <v>429</v>
       </c>
     </row>
-    <row r="33" spans="1:9">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>41</v>
       </c>
@@ -10701,7 +10701,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="34" spans="1:9">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>43</v>
       </c>
@@ -10709,7 +10709,7 @@
         <v>430</v>
       </c>
     </row>
-    <row r="35" spans="1:9">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>35</v>
       </c>
@@ -10717,7 +10717,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="36" spans="1:9">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>14</v>
       </c>
@@ -10725,7 +10725,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="37" spans="1:9">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>216</v>
       </c>
@@ -10733,7 +10733,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="38" spans="1:9">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>217</v>
       </c>
@@ -10741,7 +10741,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="39" spans="1:9">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>218</v>
       </c>
@@ -10749,7 +10749,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="40" spans="1:9">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>219</v>
       </c>
@@ -10757,307 +10757,307 @@
         <v>99</v>
       </c>
     </row>
-    <row r="41" spans="1:9">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="42" spans="1:9">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="43" spans="1:9">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="44" spans="1:9">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="45" spans="1:9">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="46" spans="1:9">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="1:9">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="48" spans="1:9">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="49" spans="1:1">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="50" spans="1:1">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="51" spans="1:1">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="52" spans="1:1">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="53" spans="1:1">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="54" spans="1:1">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="55" spans="1:1">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="56" spans="1:1">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="57" spans="1:1">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>229</v>
       </c>
     </row>
-    <row r="58" spans="1:1">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>230</v>
       </c>
     </row>
-    <row r="59" spans="1:1">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="60" spans="1:1">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="61" spans="1:1">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="62" spans="1:1">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="63" spans="1:1">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="64" spans="1:1">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="65" spans="1:1">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="66" spans="1:1">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="67" spans="1:1">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="68" spans="1:1">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="69" spans="1:1">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="70" spans="1:1">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="71" spans="1:1">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="72" spans="1:1">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="73" spans="1:1">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="74" spans="1:1">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="75" spans="1:1">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="76" spans="1:1">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="77" spans="1:1">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="78" spans="1:1">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="79" spans="1:1">
+    <row r="79" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="80" spans="1:1">
+    <row r="80" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="81" spans="1:1">
+    <row r="81" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="82" spans="1:1">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="83" spans="1:1">
+    <row r="83" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="84" spans="1:1">
+    <row r="84" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="85" spans="1:1">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="86" spans="1:1">
+    <row r="86" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="87" spans="1:1">
+    <row r="87" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="88" spans="1:1">
+    <row r="88" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="89" spans="1:1">
+    <row r="89" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A89" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="90" spans="1:1">
+    <row r="90" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A90" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="91" spans="1:1">
+    <row r="91" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A91" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="92" spans="1:1">
+    <row r="92" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A92" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="93" spans="1:1">
+    <row r="93" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A93" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="94" spans="1:1">
+    <row r="94" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A94" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="95" spans="1:1">
+    <row r="95" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A95" t="s">
         <v>245</v>
       </c>
     </row>
-    <row r="96" spans="1:1">
+    <row r="96" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A96" t="s">
         <v>246</v>
       </c>
     </row>
-    <row r="97" spans="1:1">
+    <row r="97" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A97" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="98" spans="1:1">
+    <row r="98" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A98" t="s">
         <v>248</v>
       </c>
     </row>
-    <row r="99" spans="1:1">
+    <row r="99" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A99" t="s">
         <v>249</v>
       </c>
     </row>
-    <row r="100" spans="1:1">
+    <row r="100" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A100" t="s">
         <v>250</v>
       </c>
     </row>
-    <row r="101" spans="1:1">
+    <row r="101" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A101" t="s">
         <v>251</v>
       </c>
@@ -11069,4 +11069,10 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{101ce67d-13f2-447a-bb65-0989b89dfdb4}" enabled="0" method="" siteId="{101ce67d-13f2-447a-bb65-0989b89dfdb4}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
actu 2198 a fa6
</commit_message>
<xml_diff>
--- a/backend/data/AutomatedLines.xlsx
+++ b/backend/data/AutomatedLines.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kochind-my.sharepoint.com/personal/moises_ramirez1_molex_com/Documents/aplicacionWeb/WebAppLineFinder/backend/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="654" documentId="13_ncr:1_{9CF0DDEB-C0A7-4BC9-A395-14399483BEE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFD0ED34-7814-4203-AC5A-E0ABCAD236EB}"/>
+  <xr:revisionPtr revIDLastSave="657" documentId="13_ncr:1_{9CF0DDEB-C0A7-4BC9-A395-14399483BEE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37950635-E1F0-4E91-AC26-E78B0610EA1E}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -1708,7 +1708,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1792,6 +1792,7 @@
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2066,775 +2067,6 @@
         </left>
         <right style="thin">
           <color theme="4" tint="0.39997558519241921"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color auto="1"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="none"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
         </right>
         <top/>
         <bottom/>
@@ -2996,6 +2228,775 @@
         <bottom/>
       </border>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color auto="1"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color auto="1"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color auto="1"/>
+        </left>
+        <right style="thin">
+          <color auto="1"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
   <extLst>
@@ -3010,130 +3011,130 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CECFD1AD-A5A3-4ACE-B164-6FDF2FE2E95A}" name="Tabla1" displayName="Tabla1" ref="A1:H230" totalsRowShown="0" headerRowDxfId="126" dataDxfId="125">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CECFD1AD-A5A3-4ACE-B164-6FDF2FE2E95A}" name="Tabla1" displayName="Tabla1" ref="A1:H230" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G230">
     <sortCondition ref="A118:A230"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{529D4B34-4DA7-4DEA-82D6-FD2BD15A630D}" name="Col 1" dataDxfId="124"/>
-    <tableColumn id="7" xr3:uid="{CF499674-C182-4560-8B41-0E78F331A415}" name="Col 12" dataDxfId="123"/>
-    <tableColumn id="2" xr3:uid="{45F9BB40-479B-43A5-863C-7DF090960010}" name="Col 2" dataDxfId="122"/>
-    <tableColumn id="3" xr3:uid="{35AC3272-E32E-4533-B684-783CFFC3D97D}" name="Col 3" dataDxfId="121"/>
-    <tableColumn id="4" xr3:uid="{009711B2-C3BC-4C66-A5C8-5E23732ACEC7}" name="Col 4" dataDxfId="120"/>
-    <tableColumn id="5" xr3:uid="{DBF11C8B-3BA2-4B93-8B9D-B2B98230B63B}" name="Col 5" dataDxfId="119"/>
-    <tableColumn id="6" xr3:uid="{CC41153B-24E7-4D38-B346-9455226D8193}" name="Col 6" dataDxfId="118"/>
-    <tableColumn id="8" xr3:uid="{5BD831E8-A1B8-48E7-A7CD-262D4CCFAEA7}" name="Col 7" dataDxfId="117"/>
+    <tableColumn id="1" xr3:uid="{529D4B34-4DA7-4DEA-82D6-FD2BD15A630D}" name="Col 1" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{CF499674-C182-4560-8B41-0E78F331A415}" name="Col 12" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{45F9BB40-479B-43A5-863C-7DF090960010}" name="Col 2" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{35AC3272-E32E-4533-B684-783CFFC3D97D}" name="Col 3" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{009711B2-C3BC-4C66-A5C8-5E23732ACEC7}" name="Col 4" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{DBF11C8B-3BA2-4B93-8B9D-B2B98230B63B}" name="Col 5" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{CC41153B-24E7-4D38-B346-9455226D8193}" name="Col 6" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{5BD831E8-A1B8-48E7-A7CD-262D4CCFAEA7}" name="Col 7" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2551586D-350A-4849-A83B-B0EC7C8A022F}" name="Tabla2" displayName="Tabla2" ref="A1:CX10" totalsRowShown="0" headerRowDxfId="116" dataDxfId="114" headerRowBorderDxfId="115" tableBorderDxfId="113">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2551586D-350A-4849-A83B-B0EC7C8A022F}" name="Tabla2" displayName="Tabla2" ref="A1:CX10" totalsRowShown="0" headerRowDxfId="126" dataDxfId="124" headerRowBorderDxfId="125" tableBorderDxfId="123">
   <autoFilter ref="A1:CX10" xr:uid="{2551586D-350A-4849-A83B-B0EC7C8A022F}"/>
   <tableColumns count="102">
-    <tableColumn id="1" xr3:uid="{515ED9AD-2115-402D-A669-A7974119647C}" name="Col 1" dataDxfId="112"/>
-    <tableColumn id="2" xr3:uid="{4DD548BB-E585-4E18-BEB7-EC341F80577A}" name="Col 2" dataDxfId="111"/>
-    <tableColumn id="3" xr3:uid="{7D0A8B13-FDE9-43BD-B3DD-86603D1467E1}" name="Col 3" dataDxfId="110"/>
-    <tableColumn id="4" xr3:uid="{E6CD9477-D3FD-4183-B5C5-BA5552768D31}" name="Col 4" dataDxfId="109"/>
-    <tableColumn id="5" xr3:uid="{777800CA-01CA-4618-9E1F-B70C83DAEB01}" name="Col 5" dataDxfId="108"/>
-    <tableColumn id="6" xr3:uid="{E1C1DB5D-C27D-4C23-81E5-A9DF13A78A10}" name="Col 6" dataDxfId="107"/>
-    <tableColumn id="7" xr3:uid="{47605FA4-FEAF-4F2B-B1E3-14688AA5FE34}" name="Col 7" dataDxfId="106"/>
-    <tableColumn id="8" xr3:uid="{7FDAAA4E-ACAA-47E2-89B0-2A9A7E833B2E}" name="Col 8" dataDxfId="105"/>
-    <tableColumn id="9" xr3:uid="{E85CCC77-207F-4C47-B0CB-63A4D776409B}" name="Col 9" dataDxfId="104"/>
-    <tableColumn id="10" xr3:uid="{D9D92095-084F-4C5D-AF7C-C0C0A97EF0F3}" name="Col 10" dataDxfId="103"/>
-    <tableColumn id="11" xr3:uid="{A887ACE6-719B-47C5-ADC9-25C62650ADAD}" name="Col 11" dataDxfId="102"/>
-    <tableColumn id="12" xr3:uid="{30EEE989-5F4F-491A-B3DF-CCA8797CB49A}" name="Col 12" dataDxfId="101"/>
-    <tableColumn id="13" xr3:uid="{C9FCE6BD-5206-4F1D-8C10-D352EDF4BEC0}" name="Col 13" dataDxfId="100"/>
-    <tableColumn id="14" xr3:uid="{8E498461-0417-42FB-9E0F-D7DA3B1EA813}" name="Col 14" dataDxfId="99"/>
-    <tableColumn id="15" xr3:uid="{08EDDC5C-A7C3-4E14-A3D9-A2F9DB0F3BB1}" name="Col 15" dataDxfId="98"/>
-    <tableColumn id="16" xr3:uid="{AD9AE0D2-238B-424D-9B24-07BE7442E04F}" name="Col 16" dataDxfId="97"/>
-    <tableColumn id="17" xr3:uid="{2630B814-8919-4868-8DCE-1F2573BBC5B0}" name="Col 17" dataDxfId="96"/>
-    <tableColumn id="18" xr3:uid="{03CEE4E1-31A2-4724-A645-465CD2E045B9}" name="Col 18" dataDxfId="95"/>
-    <tableColumn id="19" xr3:uid="{36A35601-EAB7-4AB7-A614-7F8935936E6A}" name="Col 19" dataDxfId="94"/>
-    <tableColumn id="20" xr3:uid="{B07CF123-370C-4A46-A187-E8C3ECA28E61}" name="Col 20" dataDxfId="93"/>
-    <tableColumn id="21" xr3:uid="{3304A7B5-755F-4660-9241-F6EF4764F80B}" name="Col 21" dataDxfId="92"/>
-    <tableColumn id="22" xr3:uid="{4D5DD45C-EB23-4740-B7A8-ECA40874A151}" name="Col 22" dataDxfId="91"/>
-    <tableColumn id="23" xr3:uid="{76D5E9A0-768E-4FE8-83FA-EFEA599A0D33}" name="Col 23" dataDxfId="90"/>
-    <tableColumn id="24" xr3:uid="{02CD437C-7E42-4463-9013-107702C2B97F}" name="Col 24" dataDxfId="89"/>
-    <tableColumn id="25" xr3:uid="{DA504FA1-64F2-4573-B961-EE7FF96F946F}" name="Col 25" dataDxfId="88"/>
-    <tableColumn id="26" xr3:uid="{080C36A3-1279-43B3-9886-9F422C5195C2}" name="Col 26" dataDxfId="87"/>
-    <tableColumn id="27" xr3:uid="{F8545C41-9CAC-4EF7-BC34-973BAA53030F}" name="Col 27" dataDxfId="86"/>
-    <tableColumn id="28" xr3:uid="{75A7CF96-CABF-47B4-AB82-4FA4E53D81FB}" name="Col 28" dataDxfId="85"/>
-    <tableColumn id="29" xr3:uid="{8172C106-C018-4748-AA79-930FD33FB140}" name="Col 29" dataDxfId="84"/>
-    <tableColumn id="30" xr3:uid="{033ADE97-F3E4-4DA3-A83E-6147BDDBF1DF}" name="Col 30" dataDxfId="83"/>
-    <tableColumn id="31" xr3:uid="{F0C16803-0361-4D9C-9477-8426659282FD}" name="Col 31" dataDxfId="82"/>
-    <tableColumn id="32" xr3:uid="{910E3D06-6155-47EA-AF66-C13FA37B096F}" name="Col 32" dataDxfId="81"/>
-    <tableColumn id="33" xr3:uid="{BCA777C5-ED01-42A4-B051-4D833909B50A}" name="Col 33" dataDxfId="80"/>
-    <tableColumn id="34" xr3:uid="{7E1688F6-81EC-4DB2-816D-DCA58D556069}" name="Col 34" dataDxfId="79"/>
-    <tableColumn id="35" xr3:uid="{A7E1220E-D975-406D-948D-AD5ED3987172}" name="Col 35" dataDxfId="78"/>
-    <tableColumn id="36" xr3:uid="{CF7860C2-B04E-4553-8766-8D2252498B7D}" name="Col 36" dataDxfId="77"/>
-    <tableColumn id="37" xr3:uid="{FD24E187-D4BD-42A0-BC83-FCE2168C419B}" name="Col 37" dataDxfId="76"/>
-    <tableColumn id="38" xr3:uid="{78753972-0217-42B3-BB8C-339E763C03E9}" name="Col 38" dataDxfId="75"/>
-    <tableColumn id="39" xr3:uid="{49D7CC7C-78D2-499D-BF5B-204884E5C2CF}" name="Col 39" dataDxfId="74"/>
-    <tableColumn id="40" xr3:uid="{1664C61D-9B35-444D-856A-B5569FE7963E}" name="Col 40" dataDxfId="73"/>
-    <tableColumn id="41" xr3:uid="{1B7B38E0-6D44-4574-B87F-DB9CB0430C27}" name="Col 41" dataDxfId="72"/>
-    <tableColumn id="42" xr3:uid="{BE1E50E5-6C10-40D3-8355-68B05DE1AE9E}" name="Col 42" dataDxfId="71"/>
-    <tableColumn id="43" xr3:uid="{F25328DB-7EF2-4D70-B37F-946281B2D9BE}" name="Col 43" dataDxfId="70"/>
-    <tableColumn id="44" xr3:uid="{E46135CD-3747-49F8-A2C5-A9F3FA2A2F15}" name="Col 44" dataDxfId="69"/>
-    <tableColumn id="45" xr3:uid="{57F610BB-9B06-403D-A345-30B797486F2A}" name="Col 45" dataDxfId="68"/>
-    <tableColumn id="46" xr3:uid="{C35D3A15-1050-4B13-A99B-A8A95FD132F0}" name="Col 46" dataDxfId="67"/>
-    <tableColumn id="47" xr3:uid="{AE1CABF3-800E-4D52-B471-5594A79A1178}" name="Col 47" dataDxfId="66"/>
-    <tableColumn id="48" xr3:uid="{33E1DF5E-0C16-42C2-82D8-059D81FB61EF}" name="Col 48" dataDxfId="65"/>
-    <tableColumn id="49" xr3:uid="{110C8421-8763-4958-BCAB-586759DB96CF}" name="Col 49" dataDxfId="64"/>
-    <tableColumn id="50" xr3:uid="{EDE7C4F3-B0A2-4507-A2E3-7B8927DB17FF}" name="Col 50" dataDxfId="63"/>
-    <tableColumn id="51" xr3:uid="{03EA894E-E948-49F6-AC7B-1339E04F49F8}" name="Col 51" dataDxfId="62"/>
-    <tableColumn id="52" xr3:uid="{D95496CB-D58F-450B-B253-10F8B3315214}" name="Col 52" dataDxfId="61"/>
-    <tableColumn id="53" xr3:uid="{88D88FC3-D469-4679-AEED-690D6BDD1563}" name="Col 53" dataDxfId="60"/>
-    <tableColumn id="54" xr3:uid="{C9F66062-BDC8-403F-9A8B-3F6CB3D9346C}" name="Col 54" dataDxfId="59"/>
-    <tableColumn id="55" xr3:uid="{FED3AF10-DE5D-4DF5-A902-80BDE81919E0}" name="Col 55" dataDxfId="58"/>
-    <tableColumn id="56" xr3:uid="{2690A48E-9EA1-41A9-9B2B-3FDF4AFAD223}" name="Col 56" dataDxfId="57"/>
-    <tableColumn id="57" xr3:uid="{D2B40034-FF19-4BF8-B181-D750E9D1A041}" name="Col 57" dataDxfId="56"/>
-    <tableColumn id="58" xr3:uid="{1404B02A-959B-456B-98DA-FC7EDEC52138}" name="Col 58" dataDxfId="55"/>
-    <tableColumn id="59" xr3:uid="{43716E72-7E67-43AB-801F-D9C41994E8E6}" name="Col 59" dataDxfId="54"/>
-    <tableColumn id="60" xr3:uid="{528A42A9-5816-468C-B2A7-1081692BFFB7}" name="Col 60" dataDxfId="53"/>
-    <tableColumn id="61" xr3:uid="{C22372D4-C12E-4487-B962-F7E4F9836534}" name="Col 61" dataDxfId="52"/>
-    <tableColumn id="62" xr3:uid="{28D784EB-BF9D-429D-A5E8-D4329D65201A}" name="Col 62" dataDxfId="51"/>
-    <tableColumn id="63" xr3:uid="{8FA59AD3-BDFE-41ED-B471-076755538EAC}" name="Col 63" dataDxfId="50"/>
-    <tableColumn id="64" xr3:uid="{AF2A2D6D-4529-48ED-A9D9-25E566D21C68}" name="Col 64" dataDxfId="49"/>
-    <tableColumn id="65" xr3:uid="{83FBFC62-D5D2-4A46-9149-ED1B85FCBC17}" name="Col 65" dataDxfId="48"/>
-    <tableColumn id="66" xr3:uid="{02788A26-6698-4416-BC3D-C7DEF6B5B6B4}" name="Col 66" dataDxfId="47"/>
-    <tableColumn id="67" xr3:uid="{41235750-E626-4FED-9EA1-42BD8F578D29}" name="Col 67" dataDxfId="46"/>
-    <tableColumn id="68" xr3:uid="{2DF4E672-C2E5-49F4-8FE8-8F563C2E74A0}" name="Col 68" dataDxfId="45"/>
-    <tableColumn id="69" xr3:uid="{45CBB860-0CF4-430A-9D41-DEDC6D4435AD}" name="Col 69" dataDxfId="44"/>
-    <tableColumn id="70" xr3:uid="{FA638996-E077-437A-AEC9-761FB83B74A8}" name="Col 70" dataDxfId="43"/>
-    <tableColumn id="71" xr3:uid="{EC0D9C98-7817-4D2F-BBF6-93E2737118F4}" name="Col 71" dataDxfId="42"/>
-    <tableColumn id="72" xr3:uid="{DA4E9A3B-364C-4787-922E-47CFDD1D23B8}" name="Col 72" dataDxfId="41"/>
-    <tableColumn id="73" xr3:uid="{6686A209-D8A9-4E28-B764-82A2AD26DD72}" name="Col 73" dataDxfId="40"/>
-    <tableColumn id="74" xr3:uid="{A97309D3-1AEB-4303-9733-6B03D92DC450}" name="Col 74" dataDxfId="39"/>
-    <tableColumn id="75" xr3:uid="{BC424F0B-0CBC-46CA-9D43-49C5D4D12084}" name="Col 75" dataDxfId="38"/>
-    <tableColumn id="76" xr3:uid="{40FFB765-2CF6-4F36-8FB4-144ABFB67BD2}" name="Col 76" dataDxfId="37"/>
-    <tableColumn id="77" xr3:uid="{4739DE29-84E8-475D-818B-7049D885DC76}" name="Col 77" dataDxfId="36"/>
-    <tableColumn id="78" xr3:uid="{7F3F3930-1E9D-45AE-ACAD-B8835C519E36}" name="Col 78" dataDxfId="35"/>
-    <tableColumn id="79" xr3:uid="{C5F83322-36B9-471A-BCD8-8CCE63CE4CC9}" name="Col 79" dataDxfId="34"/>
-    <tableColumn id="80" xr3:uid="{0AE29E9F-22FE-4103-85D1-3ED27F1C21B0}" name="Col 80" dataDxfId="33"/>
-    <tableColumn id="81" xr3:uid="{B86D5E9E-38C1-40FD-A0A0-65F8B0627EFC}" name="Col 81" dataDxfId="32"/>
-    <tableColumn id="82" xr3:uid="{DCB2BC17-B8D5-4EE9-8D35-E9333DA85146}" name="Col 82" dataDxfId="31"/>
-    <tableColumn id="83" xr3:uid="{CE75F411-AF0C-4F05-8569-EC5890BBE475}" name="Col 83" dataDxfId="30"/>
-    <tableColumn id="84" xr3:uid="{5C42F387-A9E2-4DC0-BE8D-DC5C590D89D3}" name="Col 84" dataDxfId="29"/>
-    <tableColumn id="85" xr3:uid="{29C9A99E-A5B0-40A4-AE16-4E91D03A520F}" name="Col 85" dataDxfId="28"/>
-    <tableColumn id="86" xr3:uid="{DD1E90CC-744B-40C6-AF6B-C27D715B7028}" name="Col 86" dataDxfId="27"/>
-    <tableColumn id="87" xr3:uid="{B3FCB1DB-E744-4C30-A492-F70B45EB645F}" name="Col 87" dataDxfId="26"/>
-    <tableColumn id="88" xr3:uid="{86C3CE83-2701-497E-BAAB-BD6E5BE9D25F}" name="Col 88" dataDxfId="25"/>
-    <tableColumn id="89" xr3:uid="{54E1ABF7-C9B0-4DF3-936F-B06C61F4D1AF}" name="Col 89" dataDxfId="24"/>
-    <tableColumn id="90" xr3:uid="{2F8BC889-9706-413E-8B0A-8CB66FA56EE6}" name="Col 90" dataDxfId="23"/>
-    <tableColumn id="91" xr3:uid="{744DB11E-AB2C-41E5-846F-71432CBD81E7}" name="Col 91" dataDxfId="22"/>
-    <tableColumn id="92" xr3:uid="{E9F7DAA5-0516-44B3-A6A4-DA2211281BE1}" name="Col 92" dataDxfId="21"/>
-    <tableColumn id="93" xr3:uid="{9889A6EF-A74B-423D-BDF9-A39020570EAB}" name="Col 93" dataDxfId="20"/>
-    <tableColumn id="94" xr3:uid="{540A74DA-B0E2-44FE-AE26-A7CFE9D5167A}" name="Col 94" dataDxfId="19"/>
-    <tableColumn id="95" xr3:uid="{64B11637-83D7-4E06-A33A-59DA71A9C1B1}" name="Col 95" dataDxfId="18"/>
-    <tableColumn id="96" xr3:uid="{6A83FE22-16AD-4DB7-84DC-DB55D967851C}" name="Col 96" dataDxfId="17"/>
-    <tableColumn id="97" xr3:uid="{C3E53C3E-EF93-4DF5-89F3-4B5535A4B63F}" name="Col 97" dataDxfId="16"/>
-    <tableColumn id="98" xr3:uid="{DB7106AA-4F3A-492C-B1E6-6605F7A5AFFA}" name="Col 98" dataDxfId="15"/>
-    <tableColumn id="99" xr3:uid="{092A0299-48D1-4BF5-8176-E19BBB43288F}" name="Col 99" dataDxfId="14"/>
-    <tableColumn id="100" xr3:uid="{A85ACC83-4078-4DD2-812A-10CF55A6E678}" name="Col 100" dataDxfId="13"/>
-    <tableColumn id="101" xr3:uid="{9DF18404-F344-4718-98A8-ED34BE772269}" name="Col 101" dataDxfId="12"/>
-    <tableColumn id="102" xr3:uid="{EC091E45-98D0-445E-8564-9D521EDB27CE}" name="Col 102" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{515ED9AD-2115-402D-A669-A7974119647C}" name="Col 1" dataDxfId="122"/>
+    <tableColumn id="2" xr3:uid="{4DD548BB-E585-4E18-BEB7-EC341F80577A}" name="Col 2" dataDxfId="121"/>
+    <tableColumn id="3" xr3:uid="{7D0A8B13-FDE9-43BD-B3DD-86603D1467E1}" name="Col 3" dataDxfId="120"/>
+    <tableColumn id="4" xr3:uid="{E6CD9477-D3FD-4183-B5C5-BA5552768D31}" name="Col 4" dataDxfId="119"/>
+    <tableColumn id="5" xr3:uid="{777800CA-01CA-4618-9E1F-B70C83DAEB01}" name="Col 5" dataDxfId="118"/>
+    <tableColumn id="6" xr3:uid="{E1C1DB5D-C27D-4C23-81E5-A9DF13A78A10}" name="Col 6" dataDxfId="117"/>
+    <tableColumn id="7" xr3:uid="{47605FA4-FEAF-4F2B-B1E3-14688AA5FE34}" name="Col 7" dataDxfId="116"/>
+    <tableColumn id="8" xr3:uid="{7FDAAA4E-ACAA-47E2-89B0-2A9A7E833B2E}" name="Col 8" dataDxfId="115"/>
+    <tableColumn id="9" xr3:uid="{E85CCC77-207F-4C47-B0CB-63A4D776409B}" name="Col 9" dataDxfId="114"/>
+    <tableColumn id="10" xr3:uid="{D9D92095-084F-4C5D-AF7C-C0C0A97EF0F3}" name="Col 10" dataDxfId="113"/>
+    <tableColumn id="11" xr3:uid="{A887ACE6-719B-47C5-ADC9-25C62650ADAD}" name="Col 11" dataDxfId="112"/>
+    <tableColumn id="12" xr3:uid="{30EEE989-5F4F-491A-B3DF-CCA8797CB49A}" name="Col 12" dataDxfId="111"/>
+    <tableColumn id="13" xr3:uid="{C9FCE6BD-5206-4F1D-8C10-D352EDF4BEC0}" name="Col 13" dataDxfId="110"/>
+    <tableColumn id="14" xr3:uid="{8E498461-0417-42FB-9E0F-D7DA3B1EA813}" name="Col 14" dataDxfId="109"/>
+    <tableColumn id="15" xr3:uid="{08EDDC5C-A7C3-4E14-A3D9-A2F9DB0F3BB1}" name="Col 15" dataDxfId="108"/>
+    <tableColumn id="16" xr3:uid="{AD9AE0D2-238B-424D-9B24-07BE7442E04F}" name="Col 16" dataDxfId="107"/>
+    <tableColumn id="17" xr3:uid="{2630B814-8919-4868-8DCE-1F2573BBC5B0}" name="Col 17" dataDxfId="106"/>
+    <tableColumn id="18" xr3:uid="{03CEE4E1-31A2-4724-A645-465CD2E045B9}" name="Col 18" dataDxfId="105"/>
+    <tableColumn id="19" xr3:uid="{36A35601-EAB7-4AB7-A614-7F8935936E6A}" name="Col 19" dataDxfId="104"/>
+    <tableColumn id="20" xr3:uid="{B07CF123-370C-4A46-A187-E8C3ECA28E61}" name="Col 20" dataDxfId="103"/>
+    <tableColumn id="21" xr3:uid="{3304A7B5-755F-4660-9241-F6EF4764F80B}" name="Col 21" dataDxfId="102"/>
+    <tableColumn id="22" xr3:uid="{4D5DD45C-EB23-4740-B7A8-ECA40874A151}" name="Col 22" dataDxfId="101"/>
+    <tableColumn id="23" xr3:uid="{76D5E9A0-768E-4FE8-83FA-EFEA599A0D33}" name="Col 23" dataDxfId="100"/>
+    <tableColumn id="24" xr3:uid="{02CD437C-7E42-4463-9013-107702C2B97F}" name="Col 24" dataDxfId="99"/>
+    <tableColumn id="25" xr3:uid="{DA504FA1-64F2-4573-B961-EE7FF96F946F}" name="Col 25" dataDxfId="98"/>
+    <tableColumn id="26" xr3:uid="{080C36A3-1279-43B3-9886-9F422C5195C2}" name="Col 26" dataDxfId="97"/>
+    <tableColumn id="27" xr3:uid="{F8545C41-9CAC-4EF7-BC34-973BAA53030F}" name="Col 27" dataDxfId="96"/>
+    <tableColumn id="28" xr3:uid="{75A7CF96-CABF-47B4-AB82-4FA4E53D81FB}" name="Col 28" dataDxfId="95"/>
+    <tableColumn id="29" xr3:uid="{8172C106-C018-4748-AA79-930FD33FB140}" name="Col 29" dataDxfId="94"/>
+    <tableColumn id="30" xr3:uid="{033ADE97-F3E4-4DA3-A83E-6147BDDBF1DF}" name="Col 30" dataDxfId="93"/>
+    <tableColumn id="31" xr3:uid="{F0C16803-0361-4D9C-9477-8426659282FD}" name="Col 31" dataDxfId="92"/>
+    <tableColumn id="32" xr3:uid="{910E3D06-6155-47EA-AF66-C13FA37B096F}" name="Col 32" dataDxfId="91"/>
+    <tableColumn id="33" xr3:uid="{BCA777C5-ED01-42A4-B051-4D833909B50A}" name="Col 33" dataDxfId="90"/>
+    <tableColumn id="34" xr3:uid="{7E1688F6-81EC-4DB2-816D-DCA58D556069}" name="Col 34" dataDxfId="89"/>
+    <tableColumn id="35" xr3:uid="{A7E1220E-D975-406D-948D-AD5ED3987172}" name="Col 35" dataDxfId="88"/>
+    <tableColumn id="36" xr3:uid="{CF7860C2-B04E-4553-8766-8D2252498B7D}" name="Col 36" dataDxfId="87"/>
+    <tableColumn id="37" xr3:uid="{FD24E187-D4BD-42A0-BC83-FCE2168C419B}" name="Col 37" dataDxfId="86"/>
+    <tableColumn id="38" xr3:uid="{78753972-0217-42B3-BB8C-339E763C03E9}" name="Col 38" dataDxfId="85"/>
+    <tableColumn id="39" xr3:uid="{49D7CC7C-78D2-499D-BF5B-204884E5C2CF}" name="Col 39" dataDxfId="84"/>
+    <tableColumn id="40" xr3:uid="{1664C61D-9B35-444D-856A-B5569FE7963E}" name="Col 40" dataDxfId="83"/>
+    <tableColumn id="41" xr3:uid="{1B7B38E0-6D44-4574-B87F-DB9CB0430C27}" name="Col 41" dataDxfId="82"/>
+    <tableColumn id="42" xr3:uid="{BE1E50E5-6C10-40D3-8355-68B05DE1AE9E}" name="Col 42" dataDxfId="81"/>
+    <tableColumn id="43" xr3:uid="{F25328DB-7EF2-4D70-B37F-946281B2D9BE}" name="Col 43" dataDxfId="80"/>
+    <tableColumn id="44" xr3:uid="{E46135CD-3747-49F8-A2C5-A9F3FA2A2F15}" name="Col 44" dataDxfId="79"/>
+    <tableColumn id="45" xr3:uid="{57F610BB-9B06-403D-A345-30B797486F2A}" name="Col 45" dataDxfId="78"/>
+    <tableColumn id="46" xr3:uid="{C35D3A15-1050-4B13-A99B-A8A95FD132F0}" name="Col 46" dataDxfId="77"/>
+    <tableColumn id="47" xr3:uid="{AE1CABF3-800E-4D52-B471-5594A79A1178}" name="Col 47" dataDxfId="76"/>
+    <tableColumn id="48" xr3:uid="{33E1DF5E-0C16-42C2-82D8-059D81FB61EF}" name="Col 48" dataDxfId="75"/>
+    <tableColumn id="49" xr3:uid="{110C8421-8763-4958-BCAB-586759DB96CF}" name="Col 49" dataDxfId="74"/>
+    <tableColumn id="50" xr3:uid="{EDE7C4F3-B0A2-4507-A2E3-7B8927DB17FF}" name="Col 50" dataDxfId="73"/>
+    <tableColumn id="51" xr3:uid="{03EA894E-E948-49F6-AC7B-1339E04F49F8}" name="Col 51" dataDxfId="72"/>
+    <tableColumn id="52" xr3:uid="{D95496CB-D58F-450B-B253-10F8B3315214}" name="Col 52" dataDxfId="71"/>
+    <tableColumn id="53" xr3:uid="{88D88FC3-D469-4679-AEED-690D6BDD1563}" name="Col 53" dataDxfId="70"/>
+    <tableColumn id="54" xr3:uid="{C9F66062-BDC8-403F-9A8B-3F6CB3D9346C}" name="Col 54" dataDxfId="69"/>
+    <tableColumn id="55" xr3:uid="{FED3AF10-DE5D-4DF5-A902-80BDE81919E0}" name="Col 55" dataDxfId="68"/>
+    <tableColumn id="56" xr3:uid="{2690A48E-9EA1-41A9-9B2B-3FDF4AFAD223}" name="Col 56" dataDxfId="67"/>
+    <tableColumn id="57" xr3:uid="{D2B40034-FF19-4BF8-B181-D750E9D1A041}" name="Col 57" dataDxfId="66"/>
+    <tableColumn id="58" xr3:uid="{1404B02A-959B-456B-98DA-FC7EDEC52138}" name="Col 58" dataDxfId="65"/>
+    <tableColumn id="59" xr3:uid="{43716E72-7E67-43AB-801F-D9C41994E8E6}" name="Col 59" dataDxfId="64"/>
+    <tableColumn id="60" xr3:uid="{528A42A9-5816-468C-B2A7-1081692BFFB7}" name="Col 60" dataDxfId="63"/>
+    <tableColumn id="61" xr3:uid="{C22372D4-C12E-4487-B962-F7E4F9836534}" name="Col 61" dataDxfId="62"/>
+    <tableColumn id="62" xr3:uid="{28D784EB-BF9D-429D-A5E8-D4329D65201A}" name="Col 62" dataDxfId="61"/>
+    <tableColumn id="63" xr3:uid="{8FA59AD3-BDFE-41ED-B471-076755538EAC}" name="Col 63" dataDxfId="60"/>
+    <tableColumn id="64" xr3:uid="{AF2A2D6D-4529-48ED-A9D9-25E566D21C68}" name="Col 64" dataDxfId="59"/>
+    <tableColumn id="65" xr3:uid="{83FBFC62-D5D2-4A46-9149-ED1B85FCBC17}" name="Col 65" dataDxfId="58"/>
+    <tableColumn id="66" xr3:uid="{02788A26-6698-4416-BC3D-C7DEF6B5B6B4}" name="Col 66" dataDxfId="57"/>
+    <tableColumn id="67" xr3:uid="{41235750-E626-4FED-9EA1-42BD8F578D29}" name="Col 67" dataDxfId="56"/>
+    <tableColumn id="68" xr3:uid="{2DF4E672-C2E5-49F4-8FE8-8F563C2E74A0}" name="Col 68" dataDxfId="55"/>
+    <tableColumn id="69" xr3:uid="{45CBB860-0CF4-430A-9D41-DEDC6D4435AD}" name="Col 69" dataDxfId="54"/>
+    <tableColumn id="70" xr3:uid="{FA638996-E077-437A-AEC9-761FB83B74A8}" name="Col 70" dataDxfId="53"/>
+    <tableColumn id="71" xr3:uid="{EC0D9C98-7817-4D2F-BBF6-93E2737118F4}" name="Col 71" dataDxfId="52"/>
+    <tableColumn id="72" xr3:uid="{DA4E9A3B-364C-4787-922E-47CFDD1D23B8}" name="Col 72" dataDxfId="51"/>
+    <tableColumn id="73" xr3:uid="{6686A209-D8A9-4E28-B764-82A2AD26DD72}" name="Col 73" dataDxfId="50"/>
+    <tableColumn id="74" xr3:uid="{A97309D3-1AEB-4303-9733-6B03D92DC450}" name="Col 74" dataDxfId="49"/>
+    <tableColumn id="75" xr3:uid="{BC424F0B-0CBC-46CA-9D43-49C5D4D12084}" name="Col 75" dataDxfId="48"/>
+    <tableColumn id="76" xr3:uid="{40FFB765-2CF6-4F36-8FB4-144ABFB67BD2}" name="Col 76" dataDxfId="47"/>
+    <tableColumn id="77" xr3:uid="{4739DE29-84E8-475D-818B-7049D885DC76}" name="Col 77" dataDxfId="46"/>
+    <tableColumn id="78" xr3:uid="{7F3F3930-1E9D-45AE-ACAD-B8835C519E36}" name="Col 78" dataDxfId="45"/>
+    <tableColumn id="79" xr3:uid="{C5F83322-36B9-471A-BCD8-8CCE63CE4CC9}" name="Col 79" dataDxfId="44"/>
+    <tableColumn id="80" xr3:uid="{0AE29E9F-22FE-4103-85D1-3ED27F1C21B0}" name="Col 80" dataDxfId="43"/>
+    <tableColumn id="81" xr3:uid="{B86D5E9E-38C1-40FD-A0A0-65F8B0627EFC}" name="Col 81" dataDxfId="42"/>
+    <tableColumn id="82" xr3:uid="{DCB2BC17-B8D5-4EE9-8D35-E9333DA85146}" name="Col 82" dataDxfId="41"/>
+    <tableColumn id="83" xr3:uid="{CE75F411-AF0C-4F05-8569-EC5890BBE475}" name="Col 83" dataDxfId="40"/>
+    <tableColumn id="84" xr3:uid="{5C42F387-A9E2-4DC0-BE8D-DC5C590D89D3}" name="Col 84" dataDxfId="39"/>
+    <tableColumn id="85" xr3:uid="{29C9A99E-A5B0-40A4-AE16-4E91D03A520F}" name="Col 85" dataDxfId="38"/>
+    <tableColumn id="86" xr3:uid="{DD1E90CC-744B-40C6-AF6B-C27D715B7028}" name="Col 86" dataDxfId="37"/>
+    <tableColumn id="87" xr3:uid="{B3FCB1DB-E744-4C30-A492-F70B45EB645F}" name="Col 87" dataDxfId="36"/>
+    <tableColumn id="88" xr3:uid="{86C3CE83-2701-497E-BAAB-BD6E5BE9D25F}" name="Col 88" dataDxfId="35"/>
+    <tableColumn id="89" xr3:uid="{54E1ABF7-C9B0-4DF3-936F-B06C61F4D1AF}" name="Col 89" dataDxfId="34"/>
+    <tableColumn id="90" xr3:uid="{2F8BC889-9706-413E-8B0A-8CB66FA56EE6}" name="Col 90" dataDxfId="33"/>
+    <tableColumn id="91" xr3:uid="{744DB11E-AB2C-41E5-846F-71432CBD81E7}" name="Col 91" dataDxfId="32"/>
+    <tableColumn id="92" xr3:uid="{E9F7DAA5-0516-44B3-A6A4-DA2211281BE1}" name="Col 92" dataDxfId="31"/>
+    <tableColumn id="93" xr3:uid="{9889A6EF-A74B-423D-BDF9-A39020570EAB}" name="Col 93" dataDxfId="30"/>
+    <tableColumn id="94" xr3:uid="{540A74DA-B0E2-44FE-AE26-A7CFE9D5167A}" name="Col 94" dataDxfId="29"/>
+    <tableColumn id="95" xr3:uid="{64B11637-83D7-4E06-A33A-59DA71A9C1B1}" name="Col 95" dataDxfId="28"/>
+    <tableColumn id="96" xr3:uid="{6A83FE22-16AD-4DB7-84DC-DB55D967851C}" name="Col 96" dataDxfId="27"/>
+    <tableColumn id="97" xr3:uid="{C3E53C3E-EF93-4DF5-89F3-4B5535A4B63F}" name="Col 97" dataDxfId="26"/>
+    <tableColumn id="98" xr3:uid="{DB7106AA-4F3A-492C-B1E6-6605F7A5AFFA}" name="Col 98" dataDxfId="25"/>
+    <tableColumn id="99" xr3:uid="{092A0299-48D1-4BF5-8176-E19BBB43288F}" name="Col 99" dataDxfId="24"/>
+    <tableColumn id="100" xr3:uid="{A85ACC83-4078-4DD2-812A-10CF55A6E678}" name="Col 100" dataDxfId="23"/>
+    <tableColumn id="101" xr3:uid="{9DF18404-F344-4718-98A8-ED34BE772269}" name="Col 101" dataDxfId="22"/>
+    <tableColumn id="102" xr3:uid="{EC091E45-98D0-445E-8564-9D521EDB27CE}" name="Col 102" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -8609,9 +8610,6 @@
       <c r="AB6" s="34">
         <v>2154150497</v>
       </c>
-      <c r="AC6" s="34">
-        <v>2088702198</v>
-      </c>
     </row>
     <row r="7" spans="1:52" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -8849,6 +8847,9 @@
       </c>
       <c r="Z8" s="34">
         <v>2088707042</v>
+      </c>
+      <c r="AA8" s="45">
+        <v>2088702198</v>
       </c>
     </row>
     <row r="9" spans="1:52" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
se mueve modulo 1-22981-2 a fa6 donde estaba originalmente
</commit_message>
<xml_diff>
--- a/backend/data/AutomatedLines.xlsx
+++ b/backend/data/AutomatedLines.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kochind-my.sharepoint.com/personal/moises_ramirez1_molex_com/Documents/aplicacionWeb/WebAppLineFinder/backend/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="669" documentId="13_ncr:1_{9CF0DDEB-C0A7-4BC9-A395-14399483BEE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E26667D5-0832-40C8-887F-36054051C079}"/>
+  <xr:revisionPtr revIDLastSave="672" documentId="13_ncr:1_{9CF0DDEB-C0A7-4BC9-A395-14399483BEE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27879EEC-15B9-4855-9437-2938C7A410D3}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -5667,7 +5667,7 @@
         <v>29</v>
       </c>
       <c r="D197" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.35">
@@ -6896,30 +6896,27 @@
         <v>253</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>65</v>
+        <v>35</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>33</v>
+        <v>64</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>64</v>
+        <v>11</v>
       </c>
       <c r="I3" s="13" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="J3" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="K3" s="13" t="s">
         <v>9</v>
       </c>
     </row>
@@ -7229,6 +7226,9 @@
       </c>
       <c r="W7" s="13" t="s">
         <v>13</v>
+      </c>
+      <c r="X7" s="13" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="8" spans="1:102" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
se actualizan modulos para 0049 y 0052
</commit_message>
<xml_diff>
--- a/backend/data/AutomatedLines.xlsx
+++ b/backend/data/AutomatedLines.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kochind-my.sharepoint.com/personal/moises_ramirez1_molex_com/Documents/aplicacionWeb/WebAppLineFinder/backend/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="672" documentId="13_ncr:1_{9CF0DDEB-C0A7-4BC9-A395-14399483BEE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27879EEC-15B9-4855-9437-2938C7A410D3}"/>
+  <xr:revisionPtr revIDLastSave="676" documentId="13_ncr:1_{9CF0DDEB-C0A7-4BC9-A395-14399483BEE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5350212-4C34-479D-A155-B301FFBA7916}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1338" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1342" uniqueCount="397">
   <si>
     <t>Col 1</t>
   </si>
@@ -6131,7 +6131,13 @@
         <v>74</v>
       </c>
       <c r="D228" t="s">
+        <v>76</v>
+      </c>
+      <c r="E228" t="s">
         <v>108</v>
+      </c>
+      <c r="F228" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="229" spans="1:7" x14ac:dyDescent="0.35">
@@ -6168,6 +6174,12 @@
         <v>74</v>
       </c>
       <c r="D230" t="s">
+        <v>76</v>
+      </c>
+      <c r="E230" t="s">
+        <v>108</v>
+      </c>
+      <c r="F230" t="s">
         <v>110</v>
       </c>
     </row>

</xml_diff>

<commit_message>
migracion de PNs de linea 1
</commit_message>
<xml_diff>
--- a/backend/data/AutomatedLines.xlsx
+++ b/backend/data/AutomatedLines.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kochind-my.sharepoint.com/personal/moises_ramirez1_molex_com/Documents/aplicacionWeb/WebAppLineFinder/backend/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="676" documentId="13_ncr:1_{9CF0DDEB-C0A7-4BC9-A395-14399483BEE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5350212-4C34-479D-A155-B301FFBA7916}"/>
+  <xr:revisionPtr revIDLastSave="691" documentId="13_ncr:1_{9CF0DDEB-C0A7-4BC9-A395-14399483BEE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C5DAB6A-E55D-426B-9A54-4759ACBE3403}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1342" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1347" uniqueCount="397">
   <si>
     <t>Col 1</t>
   </si>
@@ -7461,14 +7461,14 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AZ11"/>
+  <dimension ref="A1:BD11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="5.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="52" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="56" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -7578,7 +7578,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="2" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>267</v>
       </c>
@@ -7644,7 +7644,7 @@
       <c r="AI2" s="9"/>
       <c r="AJ2" s="9"/>
     </row>
-    <row r="3" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>205</v>
       </c>
@@ -7751,7 +7751,7 @@
         <v>2098700189</v>
       </c>
     </row>
-    <row r="4" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>252</v>
       </c>
@@ -7807,7 +7807,7 @@
         <v>2154150715</v>
       </c>
     </row>
-    <row r="5" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>254</v>
       </c>
@@ -7875,7 +7875,7 @@
         <v>2098706085</v>
       </c>
     </row>
-    <row r="6" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>256</v>
       </c>
@@ -7961,7 +7961,7 @@
         <v>2154150497</v>
       </c>
     </row>
-    <row r="7" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>258</v>
       </c>
@@ -8118,8 +8118,20 @@
       <c r="AZ7" s="7">
         <v>2088701390</v>
       </c>
-    </row>
-    <row r="8" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="BA7" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="BB7" s="7">
+        <v>2098700305</v>
+      </c>
+      <c r="BC7" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="BD7" s="7" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="8" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>261</v>
       </c>
@@ -8202,7 +8214,7 @@
         <v>2088702198</v>
       </c>
     </row>
-    <row r="9" spans="1:52" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>263</v>
       </c>
@@ -8218,8 +8230,17 @@
       <c r="E9" s="7">
         <v>2098706085</v>
       </c>
-    </row>
-    <row r="10" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="F9" s="7">
+        <v>2098700305</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="H9" s="7">
+        <v>2098706023</v>
+      </c>
+    </row>
+    <row r="10" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>265</v>
       </c>
@@ -8244,8 +8265,14 @@
       <c r="H10" s="7">
         <v>2154170049</v>
       </c>
-    </row>
-    <row r="11" spans="1:52" x14ac:dyDescent="0.35">
+      <c r="I10" s="7" t="s">
+        <v>296</v>
+      </c>
+      <c r="J10" s="7">
+        <v>2098706023</v>
+      </c>
+    </row>
+    <row r="11" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>377</v>
       </c>

</xml_diff>

<commit_message>
2198 se vuelve a mover de linea.
</commit_message>
<xml_diff>
--- a/backend/data/AutomatedLines.xlsx
+++ b/backend/data/AutomatedLines.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kochind-my.sharepoint.com/personal/moises_ramirez1_molex_com/Documents/aplicacionWeb/WebAppLineFinder/backend/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="691" documentId="13_ncr:1_{9CF0DDEB-C0A7-4BC9-A395-14399483BEE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C5DAB6A-E55D-426B-9A54-4759ACBE3403}"/>
+  <xr:revisionPtr revIDLastSave="695" documentId="13_ncr:1_{9CF0DDEB-C0A7-4BC9-A395-14399483BEE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CE774864-E229-4531-8942-6745D2548009}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -7076,6 +7076,9 @@
       <c r="AF5" s="13" t="s">
         <v>107</v>
       </c>
+      <c r="AG5" s="13" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="6" spans="1:102" x14ac:dyDescent="0.35">
       <c r="A6" s="11" t="s">
@@ -7235,9 +7238,6 @@
       </c>
       <c r="V7" s="14" t="s">
         <v>79</v>
-      </c>
-      <c r="W7" s="13" t="s">
-        <v>13</v>
       </c>
       <c r="X7" s="13" t="s">
         <v>65</v>
@@ -7960,6 +7960,9 @@
       <c r="AB6" s="7">
         <v>2154150497</v>
       </c>
+      <c r="AC6" s="7">
+        <v>2088702198</v>
+      </c>
     </row>
     <row r="7" spans="1:56" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
@@ -8209,9 +8212,6 @@
       </c>
       <c r="Z8" s="7">
         <v>2088707042</v>
-      </c>
-      <c r="AA8" s="7">
-        <v>2088702198</v>
       </c>
     </row>
     <row r="9" spans="1:56" x14ac:dyDescent="0.35">

</xml_diff>